<commit_message>
Sync FP16 operand variation artifacts
</commit_message>
<xml_diff>
--- a/docs/experiments/fp16_energy/A100_FP16_FULL_SWEEP_TABLE.xlsx
+++ b/docs/experiments/fp16_energy/A100_FP16_FULL_SWEEP_TABLE.xlsx
@@ -60,7 +60,7 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>pJ/bit</t>
+          <t>pJ/FLOP</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Slope pJ/bit</t>
+          <t>Slope pJ/FLOP</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>t384_b4, 0.1144 +/- 0.0047 pJ/bit</t>
+          <t>t384_b4, 0.1144 +/- 0.0047 pJ/FLOP</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>t192_b8, 0.1050 +/- 0.0013 pJ/bit</t>
+          <t>t192_b8, 0.1050 +/- 0.0013 pJ/FLOP</t>
         </is>
       </c>
     </row>

</xml_diff>